<commit_message>
fix(engine): demo-eve fix wave — roster segmentation, zero-data refusal, stored packets, version badge, honest copy (F1-F5, v166)
Fixes the three capability blockers surfaced by the v0.2.65 independent test:
- F1: roster-block segmentation kills fabricated children (18→18, not 35)
- F1b: per-entry exclude in import preview (teacher safety net)
- F2: hard zero-data refusal gate in Ask — code, not prompt guidance
- F3: packet preview/print renders the STORED reviewed artifact (zero model
  calls on the print path; regenerate replaces the stored record)
- F4: app version badge in the topbar (desktop + browser mode)
- F5: import copy corrected to preview-first truth; xlsx-specific guidance

Suite: 2475 passed, 13 skipped. UI contract v166. Preflight 6/6.
Spec: dev/SPEC_LV_DEMO_EVE_FIX_2026-08-19.md
Report: dev/REPORT_LV_DEMO_EVE_FIX_2026-08-19.md

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/docpipe/synthetic-corpus/synthetic_class_list.xlsx
+++ b/tests/fixtures/docpipe/synthetic-corpus/synthetic_class_list.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -562,28 +562,150 @@
           <t>Tommaso</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1/2 groups alternate Fridays</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>1/2 groups alternate Fridays</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1/2 groups swap after break</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1/2 groups swap after break</t>
+          <t>1/2 groups for Music/Homeroom</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1/2 groups for Music/Homeroom</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Marco Bianchi</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Nora Rossi</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Giulia Riva</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Pietro Serra</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sara Conti</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Luca Ferri</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Anna (Annie) Villa</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Leo Fontana</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Elisa Greco</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tommaso Marini</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Camilla Gatti</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1/2 groups for STEAM/Homeroom</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1/2 groups for STEAM/Homeroom</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Tommaso Marini</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Elisa Greco</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Camilla Gatti</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Leo Fontana</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Luca Ferri</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sara Conti</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Anna (Annie) Villa</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Pietro Serra</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Nora Rossi</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Marco Bianchi</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Giulia Riva</t>
         </is>
       </c>
     </row>
@@ -598,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -713,27 +835,115 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1/2 groups alternate Fridays</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1/2 groups alternate Fridays</t>
-        </is>
-      </c>
-    </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1/2 groups swap after break</t>
+          <t>1/2 groups for Music/Homeroom</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1/2 groups swap after break</t>
+          <t>1/2 groups for Music/Homeroom</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Matteo Barbieri</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sofia Caruso</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Alice Monti</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Filippo Neri</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Emma Longo</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Diego Marchetti</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Viola Pellegrini</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Oscar Sanna</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1/2 groups for STEAM/Homeroom</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1/2 groups for STEAM/Homeroom</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Diego Marchetti</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Emma Longo</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Oscar Sanna</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Viola Pellegrini</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sofia Caruso</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Matteo Barbieri</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Filippo Neri</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Alice Monti</t>
         </is>
       </c>
     </row>

</xml_diff>